<commit_message>
Update CTCdata.xlsx production data
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/CTCdata.xlsx
+++ b/data/CTCdata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="13660"/>
+    <workbookView windowWidth="27660" windowHeight="13040"/>
   </bookViews>
   <sheets>
     <sheet name="Crop_production" sheetId="1" r:id="rId1"/>
@@ -1512,7 +1512,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="4">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>

</xml_diff>

<commit_message>
Add user manual, public UX, and production-ready deployment docs.
Includes Data Contribution panel, terminology tooltips, official English province names, homepage footer and valorisation highlights, moisture-corrected biochar reference table, and Streamlit Cloud public-access guidance.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/CTCdata.xlsx
+++ b/data/CTCdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhongxinzhi/Desktop/CTCv0.1/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECA2938-DE8E-4948-B157-5721900128DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF955756-9CCD-A44F-AAC4-BE3136912611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3710" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3709" uniqueCount="91">
   <si>
     <t>Year</t>
   </si>
@@ -352,9 +352,6 @@
   </si>
   <si>
     <t>Slow pyrolysis, 450℃, 30mins RT (Uni Hasselt)</t>
-  </si>
-  <si>
-    <t>\</t>
   </si>
   <si>
     <t>Slow pyrolysis, 450℃, 30mins RT (Medina et al., 2025)</t>
@@ -16356,10 +16353,10 @@
         <v>71</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>89</v>
       </c>
       <c r="F1" t="s">
         <v>72</v>
@@ -16388,7 +16385,7 @@
         <v>0.05</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G2">
         <v>0.22750000000000001</v>
@@ -16559,9 +16556,6 @@
       <c r="B10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
-        <v>81</v>
-      </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
@@ -16666,7 +16660,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G15">
         <v>0.22750000000000001</v>
@@ -16726,7 +16720,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G18">
         <v>0.22750000000000001</v>
@@ -16803,7 +16797,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>0.22750000000000001</v>
@@ -16829,7 +16823,7 @@
         <v>5.8700000000000002E-2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>0.22750000000000001</v>
@@ -16872,7 +16866,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G25">
         <v>0.22750000000000001</v>
@@ -16898,7 +16892,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G26">
         <v>0.22750000000000001</v>
@@ -16924,7 +16918,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G27">
         <v>0.22750000000000001</v>
@@ -16950,7 +16944,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G28">
         <v>0.22750000000000001</v>
@@ -16976,7 +16970,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G29">
         <v>0.22750000000000001</v>
@@ -17096,7 +17090,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G35">
         <v>0.22750000000000001</v>
@@ -17207,7 +17201,7 @@
         <v>0.08</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G41">
         <v>0.22750000000000001</v>
@@ -17250,7 +17244,7 @@
         <v>0.05</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G43">
         <v>0.22750000000000001</v>
@@ -17328,7 +17322,7 @@
         <v>7.0999999999999994E-2</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G46">
         <v>0.22750000000000001</v>
@@ -17405,7 +17399,7 @@
         <v>0.05</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G50">
         <v>0.22750000000000001</v>
@@ -17550,7 +17544,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F58" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G58">
         <v>0.22750000000000001</v>
@@ -17576,7 +17570,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F59" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G59">
         <v>0.22750000000000001</v>
@@ -17840,7 +17834,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G74">
         <v>0.22750000000000001</v>
@@ -17883,7 +17877,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G76">
         <v>0.22750000000000001</v>
@@ -17909,7 +17903,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G77">
         <v>0.22750000000000001</v>
@@ -17935,7 +17929,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G78">
         <v>0.22750000000000001</v>
@@ -17961,7 +17955,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G79">
         <v>0.22750000000000001</v>

</xml_diff>